<commit_message>
test excel and update excel column fix
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <workbookPr codeName="BuÇalışmaKitabı"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PTAReceiptParser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9910E75-7977-4848-B69A-C0FB971FF058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E626C3C8-4193-4818-AC68-C3582277F6D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{0D2934DA-576D-47CA-B498-C437B9EBB0B4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Dummy" sheetId="2" r:id="rId1"/>
-    <sheet name="TEBKrediKartı" sheetId="1" r:id="rId2"/>
+    <sheet name="Dummy" sheetId="1" r:id="rId1"/>
+    <sheet name="TEBKrediKartı" sheetId="2" r:id="rId2"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId3"/>
@@ -25,19 +25,17 @@
     <definedName name="_14.10.2022">#REF!</definedName>
     <definedName name="_19.03.2023">#REF!</definedName>
     <definedName name="_31.01.2025">[1]Bank_Info!#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">TEBKrediKartı!$A$1:$N$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">TEBKrediKartı!$A$1:$N$10</definedName>
     <definedName name="Bank_Desc.">#REF!</definedName>
     <definedName name="Borçlar_Kredi_Kartları_SHE_TEB">#REF!</definedName>
     <definedName name="DEVİR_BAKİYESİ">[1]IMPORT!#REF!</definedName>
-    <definedName name="DışVeri_1" localSheetId="1">TEBKrediKartı!$A$1:$AD$19</definedName>
+    <definedName name="DışVeri_1" localSheetId="1">TEBKrediKartı!$A$1:$AD$10</definedName>
     <definedName name="Import_Area">[1]IMPORT!#REF!</definedName>
     <definedName name="Varlıklar_Yatırım_TEB_Hisse_DMLKT">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -122,34 +120,34 @@
     <t>qd8ivwk0kx0x3hq12gaenb3ahphkqaqn</t>
   </si>
   <si>
+    <t>mn8p2wr979vnkpornu9g8hj52jsja7dx</t>
+  </si>
+  <si>
+    <t>Gelir:Kampanya</t>
+  </si>
+  <si>
+    <t>gi7uiipnlogegaxehc15k684imbam81u</t>
+  </si>
+  <si>
+    <t>Gider:Aile:Kasko/Sigorta</t>
+  </si>
+  <si>
+    <t>1coor8ctracqffj3m2xk98ailhi316hs</t>
+  </si>
+  <si>
+    <t>uf06kyt5giims4rlsbs9nu9yxtekc6ki</t>
+  </si>
+  <si>
+    <t>s2e2bx0kif1ny9hmhhywrpajdd5x7hl4</t>
+  </si>
+  <si>
+    <t>Gider:Abonelikler:Netflix</t>
+  </si>
+  <si>
+    <t>kopb3dh2a46yiac2cbw7ee2jfuah2466</t>
+  </si>
+  <si>
     <t>Gider:Market</t>
-  </si>
-  <si>
-    <t>mn8p2wr979vnkpornu9g8hj52jsja7dx</t>
-  </si>
-  <si>
-    <t>Gelir:Kampanya</t>
-  </si>
-  <si>
-    <t>gi7uiipnlogegaxehc15k684imbam81u</t>
-  </si>
-  <si>
-    <t>Gider:Aile:Kasko/Sigorta</t>
-  </si>
-  <si>
-    <t>1coor8ctracqffj3m2xk98ailhi316hs</t>
-  </si>
-  <si>
-    <t>uf06kyt5giims4rlsbs9nu9yxtekc6ki</t>
-  </si>
-  <si>
-    <t>s2e2bx0kif1ny9hmhhywrpajdd5x7hl4</t>
-  </si>
-  <si>
-    <t>Gider:Abonelikler:Netflix</t>
-  </si>
-  <si>
-    <t>kopb3dh2a46yiac2cbw7ee2jfuah2466</t>
   </si>
 </sst>
 </file>
@@ -213,9 +211,6 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="RULES"/>
       <sheetName val="Bank_Info"/>
@@ -498,7 +493,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5AEFFE0-0047-4804-BFC1-FA5422D30964}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Sayfa1"/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
@@ -507,7 +503,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B648FDDA-9EFF-402B-BC9C-05C6E5F0326E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sayfa19">
     <tabColor rgb="FFC6E0B4"/>
   </sheetPr>
@@ -525,7 +521,7 @@
     <col min="9" max="9" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.21875" customWidth="1"/>
     <col min="13" max="13" width="70.44140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="8" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="6" bestFit="1" customWidth="1"/>
@@ -680,7 +676,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>46122</v>
+        <v>46107</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>13</v>
@@ -698,7 +694,7 @@
         <v>16</v>
       </c>
       <c r="I6" s="3">
-        <v>-70</v>
+        <v>-333.07</v>
       </c>
       <c r="J6" s="2">
         <v>1</v>
@@ -709,23 +705,15 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="3">
-        <v>70</v>
-      </c>
-      <c r="J7" s="2">
-        <v>1</v>
-      </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
+      <c r="H7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7">
+        <v>333.07</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
@@ -735,7 +723,7 @@
         <v>13</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
@@ -754,7 +742,7 @@
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -765,7 +753,7 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I9" s="3">
         <v>-9.75</v>
@@ -784,7 +772,7 @@
         <v>13</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
@@ -803,7 +791,7 @@
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -814,7 +802,7 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I11" s="3">
         <v>598.78</v>
@@ -833,7 +821,7 @@
         <v>13</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
@@ -852,7 +840,7 @@
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -863,7 +851,7 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I13" s="3">
         <v>-9.75</v>
@@ -882,7 +870,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
@@ -901,7 +889,7 @@
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -912,7 +900,7 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I15" s="3">
         <v>0</v>
@@ -931,7 +919,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
@@ -950,7 +938,7 @@
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -961,7 +949,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I17" s="3">
         <v>379.99</v>
@@ -980,7 +968,7 @@
         <v>13</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
@@ -999,7 +987,7 @@
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
@@ -1010,7 +998,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="I19" s="3">
         <v>70</v>
@@ -1022,7 +1010,7 @@
       <c r="M19" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N19" xr:uid="{94A19100-6342-40C9-A5E3-4D775EC4A437}"/>
+  <autoFilter ref="A1:N10" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>